<commit_message>
feat: initialize project structure with Express server, environment configurations, documentation, and database utility modules.
</commit_message>
<xml_diff>
--- a/docs/hms-mvp-api-resource-estimation.xlsx
+++ b/docs/hms-mvp-api-resource-estimation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BrainStation 23\Healthcare Management System\project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB7E9A20-C202-47F7-A458-00280FA6724D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C20944F-A771-40EA-8A8E-E9FD1FAE69E1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="292">
   <si>
     <t>Healthcare Management System - MVP API Resource Estimation</t>
   </si>
@@ -112,12 +112,6 @@
     <t>Revoke refresh session</t>
   </si>
   <si>
-    <t>Get current authenticated user</t>
-  </si>
-  <si>
-    <t>GET /auth/me</t>
-  </si>
-  <si>
     <t>users, patient_profiles, doctor_profiles, staff_profiles</t>
   </si>
   <si>
@@ -163,9 +157,6 @@
     <t>Pagination and role/status filters</t>
   </si>
   <si>
-    <t>Create doctor/staff user</t>
-  </si>
-  <si>
     <t>POST /users</t>
   </si>
   <si>
@@ -175,9 +166,6 @@
     <t>Admin creates account and role-specific profile</t>
   </si>
   <si>
-    <t>Update user status</t>
-  </si>
-  <si>
     <t>PATCH /users/{userId}/status</t>
   </si>
   <si>
@@ -208,9 +196,6 @@
     <t>Validate demographics and basic medical fields</t>
   </si>
   <si>
-    <t>View patient details</t>
-  </si>
-  <si>
     <t>GET /patients/{patientId}</t>
   </si>
   <si>
@@ -223,9 +208,6 @@
     <t>doctors</t>
   </si>
   <si>
-    <t>List/search doctors</t>
-  </si>
-  <si>
     <t>GET /doctors</t>
   </si>
   <si>
@@ -235,9 +217,6 @@
     <t>Specialty filter and active doctor filter</t>
   </si>
   <si>
-    <t>View doctor profile</t>
-  </si>
-  <si>
     <t>GET /doctors/{doctorId}</t>
   </si>
   <si>
@@ -259,9 +238,6 @@
     <t>staff</t>
   </si>
   <si>
-    <t>List staff for admin</t>
-  </si>
-  <si>
     <t>GET /staff</t>
   </si>
   <si>
@@ -274,12 +250,6 @@
     <t>Doctor Discovery</t>
   </si>
   <si>
-    <t>appointment-slots</t>
-  </si>
-  <si>
-    <t>Calculate available slots</t>
-  </si>
-  <si>
     <t>GET /doctors/{doctorId}/available-slots</t>
   </si>
   <si>
@@ -358,9 +328,6 @@
     <t>Usually called after visit completion</t>
   </si>
   <si>
-    <t>doctor-unavailability</t>
-  </si>
-  <si>
     <t>Doctor blocks unavailable time</t>
   </si>
   <si>
@@ -899,13 +866,131 @@
   </si>
   <si>
     <t>Schema Tables (Possibly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET /auth/me </t>
+  </si>
+  <si>
+    <t xml:space="preserve">users </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Create doctor/staff user </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(Admin authorized only) </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Get current authenticated user </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(by bearer token)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Update user status </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(Admin &amp; user authorized only) </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">List staff for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>admin</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">List/search doctors </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(public)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">View patient details </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(maybe won't use)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">View doctor profile </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(public)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Calculate available slots </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(public)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -936,6 +1021,18 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1052,12 +1149,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1075,6 +1166,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1394,7 +1491,7 @@
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="42" customWidth="1"/>
@@ -1405,31 +1502,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="14" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1450,7 +1547,7 @@
         <v>6</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>7</v>
@@ -1463,7 +1560,7 @@
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B3" t="s">
@@ -1492,7 +1589,7 @@
       </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="10"/>
+      <c r="A4" s="8"/>
       <c r="B4" t="s">
         <v>11</v>
       </c>
@@ -1519,7 +1616,7 @@
       </c>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="10"/>
+      <c r="A5" s="8"/>
       <c r="B5" t="s">
         <v>11</v>
       </c>
@@ -1546,7 +1643,7 @@
       </c>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="10"/>
+      <c r="A6" s="8"/>
       <c r="B6" t="s">
         <v>11</v>
       </c>
@@ -1573,48 +1670,48 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="28.8">
-      <c r="A7" s="10"/>
+      <c r="A7" s="8"/>
       <c r="B7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>282</v>
+      </c>
+      <c r="F7" t="s">
         <v>30</v>
       </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="G7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" t="s">
         <v>31</v>
       </c>
-      <c r="F7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" t="s">
-        <v>33</v>
-      </c>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="10"/>
+      <c r="A8" s="8"/>
       <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
         <v>34</v>
       </c>
-      <c r="D8" t="s">
+      <c r="F8" t="s">
         <v>35</v>
-      </c>
-      <c r="E8" t="s">
-        <v>36</v>
-      </c>
-      <c r="F8" t="s">
-        <v>37</v>
       </c>
       <c r="G8" s="2">
         <v>2</v>
@@ -1623,22 +1720,22 @@
         <v>16</v>
       </c>
       <c r="I8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="11"/>
+      <c r="A9" s="9"/>
       <c r="B9" t="s">
         <v>11</v>
       </c>
       <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" t="s">
         <v>39</v>
-      </c>
-      <c r="D9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" t="s">
-        <v>41</v>
       </c>
       <c r="F9" t="s">
         <v>20</v>
@@ -1650,105 +1747,105 @@
         <v>16</v>
       </c>
       <c r="I9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="9" t="s">
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
         <v>43</v>
       </c>
-      <c r="B10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="F10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" t="s">
         <v>44</v>
       </c>
-      <c r="D10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" t="s">
+    </row>
+    <row r="11" spans="1:9" ht="28.8">
+      <c r="A11" s="8"/>
+      <c r="B11" t="s">
+        <v>283</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="D11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" t="s">
         <v>45</v>
       </c>
-      <c r="F10" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H10" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" t="s">
+      <c r="F11" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" ht="28.8">
-      <c r="A11" s="10"/>
-      <c r="B11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="G11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" t="s">
         <v>47</v>
       </c>
-      <c r="D11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" t="s">
+    </row>
+    <row r="12" spans="1:9" ht="28.8">
+      <c r="A12" s="8"/>
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="D12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" t="s">
         <v>48</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F12" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" t="s">
         <v>49</v>
       </c>
-      <c r="G11" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H11" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" t="s">
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="8"/>
+      <c r="B13" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="10"/>
-      <c r="B12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="C13" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D12" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="D13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" t="s">
         <v>52</v>
-      </c>
-      <c r="F12" t="s">
-        <v>37</v>
-      </c>
-      <c r="G12" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H12" t="s">
-        <v>16</v>
-      </c>
-      <c r="I12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="10"/>
-      <c r="B13" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" t="s">
-        <v>13</v>
-      </c>
-      <c r="E13" t="s">
-        <v>56</v>
       </c>
       <c r="F13" t="s">
         <v>15</v>
@@ -1760,1301 +1857,1301 @@
         <v>16</v>
       </c>
       <c r="I13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="8"/>
+      <c r="B14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H14" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="10"/>
-      <c r="B14" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" t="s">
+    <row r="15" spans="1:9">
+      <c r="A15" s="8"/>
+      <c r="B15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" t="s">
         <v>58</v>
       </c>
-      <c r="D14" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="F15" t="s">
         <v>59</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" t="s">
         <v>60</v>
       </c>
-      <c r="G14" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I14" t="s">
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="8"/>
+      <c r="B16" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15" s="10"/>
-      <c r="B15" t="s">
-        <v>54</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="C16" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" t="s">
         <v>62</v>
       </c>
-      <c r="D15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="F16" t="s">
         <v>63</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" t="s">
         <v>64</v>
       </c>
-      <c r="G15" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H15" t="s">
-        <v>16</v>
-      </c>
-      <c r="I15" t="s">
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="8"/>
+      <c r="B17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="D17" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" s="10"/>
-      <c r="B16" t="s">
+      <c r="F17" t="s">
+        <v>63</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" t="s">
         <v>66</v>
       </c>
-      <c r="C16" t="s">
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="8"/>
+      <c r="B18" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" t="s">
         <v>67</v>
       </c>
-      <c r="D16" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" t="s">
+      <c r="D18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" t="s">
         <v>68</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F18" t="s">
         <v>69</v>
       </c>
-      <c r="G16" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H16" t="s">
-        <v>16</v>
-      </c>
-      <c r="I16" t="s">
+      <c r="G18" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H18" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
-      <c r="A17" s="10"/>
-      <c r="B17" t="s">
-        <v>66</v>
-      </c>
-      <c r="C17" t="s">
+    <row r="19" spans="1:9">
+      <c r="A19" s="9"/>
+      <c r="B19" t="s">
         <v>71</v>
       </c>
-      <c r="D17" t="s">
-        <v>13</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="C19" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="D19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" t="s">
         <v>72</v>
       </c>
-      <c r="F17" t="s">
-        <v>69</v>
-      </c>
-      <c r="G17" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H17" t="s">
-        <v>16</v>
-      </c>
-      <c r="I17" t="s">
+      <c r="F19" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18" s="10"/>
-      <c r="B18" t="s">
-        <v>66</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="G19" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H19" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" t="s">
         <v>74</v>
-      </c>
-      <c r="D18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" t="s">
-        <v>75</v>
-      </c>
-      <c r="F18" t="s">
-        <v>76</v>
-      </c>
-      <c r="G18" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H18" t="s">
-        <v>16</v>
-      </c>
-      <c r="I18" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" s="11"/>
-      <c r="B19" t="s">
-        <v>78</v>
-      </c>
-      <c r="C19" t="s">
-        <v>79</v>
-      </c>
-      <c r="D19" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" t="s">
-        <v>80</v>
-      </c>
-      <c r="F19" t="s">
-        <v>81</v>
-      </c>
-      <c r="G19" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H19" t="s">
-        <v>16</v>
-      </c>
-      <c r="I19" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="28.8">
       <c r="A20" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="D20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" t="s">
+        <v>76</v>
+      </c>
+      <c r="F20" t="s">
+        <v>77</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H20" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="43.2">
+      <c r="A21" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" t="s">
+        <v>82</v>
+      </c>
+      <c r="F21" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="G21" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H21" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="5" t="s">
+    </row>
+    <row r="22" spans="1:9" ht="28.8">
+      <c r="A22" s="8"/>
+      <c r="B22" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" t="s">
         <v>85</v>
       </c>
-      <c r="D20" t="s">
-        <v>13</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="D22" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" t="s">
         <v>86</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="G20" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H20" t="s">
-        <v>16</v>
-      </c>
-      <c r="I20" t="s">
+      <c r="G22" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H22" t="s">
+        <v>16</v>
+      </c>
+      <c r="I22" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="43.2">
-      <c r="A21" s="9" t="s">
+    <row r="23" spans="1:9" ht="28.8">
+      <c r="A23" s="8"/>
+      <c r="B23" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" t="s">
         <v>89</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D23" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" t="s">
         <v>90</v>
       </c>
-      <c r="C21" t="s">
+      <c r="F23" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H23" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" t="s">
         <v>91</v>
       </c>
-      <c r="D21" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" t="s">
+    </row>
+    <row r="24" spans="1:9" ht="28.8">
+      <c r="A24" s="8"/>
+      <c r="B24" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" t="s">
         <v>92</v>
       </c>
-      <c r="F21" t="s">
+      <c r="D24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" t="s">
         <v>93</v>
       </c>
-      <c r="G21" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H21" t="s">
-        <v>16</v>
-      </c>
-      <c r="I21" t="s">
+      <c r="F24" t="s">
+        <v>87</v>
+      </c>
+      <c r="G24" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H24" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="28.8">
-      <c r="A22" s="10"/>
-      <c r="B22" t="s">
-        <v>90</v>
-      </c>
-      <c r="C22" t="s">
+    <row r="25" spans="1:9">
+      <c r="A25" s="8"/>
+      <c r="B25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" t="s">
         <v>95</v>
       </c>
-      <c r="D22" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22" t="s">
+      <c r="D25" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" t="s">
         <v>96</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F25" t="s">
+        <v>80</v>
+      </c>
+      <c r="G25" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H25" t="s">
+        <v>16</v>
+      </c>
+      <c r="I25" t="s">
         <v>97</v>
       </c>
-      <c r="G22" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H22" t="s">
-        <v>16</v>
-      </c>
-      <c r="I22" t="s">
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="8"/>
+      <c r="B26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C26" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" ht="28.8">
-      <c r="A23" s="10"/>
-      <c r="B23" t="s">
-        <v>90</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" t="s">
         <v>99</v>
       </c>
-      <c r="D23" t="s">
-        <v>13</v>
-      </c>
-      <c r="E23" t="s">
+      <c r="F26" t="s">
         <v>100</v>
       </c>
-      <c r="F23" t="s">
-        <v>97</v>
-      </c>
-      <c r="G23" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H23" t="s">
-        <v>16</v>
-      </c>
-      <c r="I23" t="s">
+      <c r="G26" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H26" t="s">
+        <v>16</v>
+      </c>
+      <c r="I26" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="28.8">
-      <c r="A24" s="10"/>
-      <c r="B24" t="s">
-        <v>90</v>
-      </c>
-      <c r="C24" t="s">
+    <row r="27" spans="1:9" ht="28.8">
+      <c r="A27" s="9"/>
+      <c r="B27" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" t="s">
         <v>102</v>
       </c>
-      <c r="D24" t="s">
-        <v>13</v>
-      </c>
-      <c r="E24" t="s">
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" t="s">
         <v>103</v>
       </c>
-      <c r="F24" t="s">
-        <v>97</v>
-      </c>
-      <c r="G24" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H24" t="s">
-        <v>16</v>
-      </c>
-      <c r="I24" t="s">
+      <c r="F27" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" s="10"/>
-      <c r="B25" t="s">
-        <v>90</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="G27" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H27" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27" t="s">
         <v>105</v>
       </c>
-      <c r="D25" t="s">
-        <v>13</v>
-      </c>
-      <c r="E25" t="s">
+    </row>
+    <row r="28" spans="1:9" ht="28.8" customHeight="1">
+      <c r="A28" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F25" t="s">
-        <v>90</v>
-      </c>
-      <c r="G25" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H25" t="s">
-        <v>16</v>
-      </c>
-      <c r="I25" t="s">
+      <c r="B28" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26" s="10"/>
-      <c r="B26" t="s">
-        <v>90</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="C28" t="s">
         <v>108</v>
       </c>
-      <c r="D26" t="s">
-        <v>13</v>
-      </c>
-      <c r="E26" t="s">
+      <c r="D28" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" t="s">
         <v>109</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F28" t="s">
         <v>110</v>
       </c>
-      <c r="G26" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I26" t="s">
+      <c r="G28" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H28" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="28.8">
-      <c r="A27" s="11"/>
-      <c r="B27" t="s">
+    <row r="29" spans="1:9">
+      <c r="A29" s="8"/>
+      <c r="B29" t="s">
+        <v>107</v>
+      </c>
+      <c r="C29" t="s">
         <v>112</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" t="s">
         <v>113</v>
       </c>
-      <c r="D27" t="s">
-        <v>13</v>
-      </c>
-      <c r="E27" t="s">
+      <c r="F29" t="s">
         <v>114</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G29" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H29" t="s">
+        <v>16</v>
+      </c>
+      <c r="I29" t="s">
         <v>115</v>
       </c>
-      <c r="G27" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H27" t="s">
-        <v>16</v>
-      </c>
-      <c r="I27" t="s">
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="8"/>
+      <c r="B30" t="s">
+        <v>107</v>
+      </c>
+      <c r="C30" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" ht="28.8" customHeight="1">
-      <c r="A28" s="9" t="s">
+      <c r="D30" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30" t="s">
         <v>117</v>
       </c>
-      <c r="B28" t="s">
+      <c r="F30" t="s">
+        <v>107</v>
+      </c>
+      <c r="G30" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H30" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" t="s">
         <v>118</v>
       </c>
-      <c r="C28" t="s">
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" s="8"/>
+      <c r="B31" t="s">
+        <v>107</v>
+      </c>
+      <c r="C31" t="s">
         <v>119</v>
       </c>
-      <c r="D28" t="s">
-        <v>13</v>
-      </c>
-      <c r="E28" t="s">
+      <c r="D31" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" t="s">
         <v>120</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G31" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H31" t="s">
+        <v>16</v>
+      </c>
+      <c r="I31" t="s">
         <v>121</v>
       </c>
-      <c r="G28" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H28" t="s">
-        <v>16</v>
-      </c>
-      <c r="I28" t="s">
+    </row>
+    <row r="32" spans="1:9" ht="28.8">
+      <c r="A32" s="8"/>
+      <c r="B32" t="s">
+        <v>107</v>
+      </c>
+      <c r="C32" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="A29" s="10"/>
-      <c r="B29" t="s">
-        <v>118</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="D32" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" t="s">
         <v>123</v>
       </c>
-      <c r="D29" t="s">
-        <v>13</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="F32" t="s">
         <v>124</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G32" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H32" t="s">
+        <v>16</v>
+      </c>
+      <c r="I32" t="s">
         <v>125</v>
       </c>
-      <c r="G29" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H29" t="s">
-        <v>16</v>
-      </c>
-      <c r="I29" t="s">
+    </row>
+    <row r="33" spans="1:9" ht="57.6">
+      <c r="A33" s="8"/>
+      <c r="B33" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="30" spans="1:9">
-      <c r="A30" s="10"/>
-      <c r="B30" t="s">
-        <v>118</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="C33" t="s">
         <v>127</v>
       </c>
-      <c r="D30" t="s">
-        <v>13</v>
-      </c>
-      <c r="E30" t="s">
+      <c r="D33" t="s">
         <v>128</v>
       </c>
-      <c r="F30" t="s">
-        <v>118</v>
-      </c>
-      <c r="G30" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H30" t="s">
-        <v>16</v>
-      </c>
-      <c r="I30" t="s">
+      <c r="E33" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="31" spans="1:9">
-      <c r="A31" s="10"/>
-      <c r="B31" t="s">
-        <v>118</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="F33" t="s">
         <v>130</v>
       </c>
-      <c r="D31" t="s">
-        <v>13</v>
-      </c>
-      <c r="E31" t="s">
+      <c r="G33" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H33" t="s">
+        <v>16</v>
+      </c>
+      <c r="I33" t="s">
         <v>131</v>
       </c>
-      <c r="F31" t="s">
-        <v>125</v>
-      </c>
-      <c r="G31" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H31" t="s">
-        <v>16</v>
-      </c>
-      <c r="I31" t="s">
+    </row>
+    <row r="34" spans="1:9" ht="28.8">
+      <c r="A34" s="8"/>
+      <c r="B34" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" ht="28.8">
-      <c r="A32" s="10"/>
-      <c r="B32" t="s">
-        <v>118</v>
-      </c>
-      <c r="C32" t="s">
+      <c r="C34" t="s">
         <v>133</v>
       </c>
-      <c r="D32" t="s">
-        <v>13</v>
-      </c>
-      <c r="E32" t="s">
+      <c r="D34" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" t="s">
         <v>134</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F34" t="s">
         <v>135</v>
       </c>
-      <c r="G32" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H32" t="s">
-        <v>16</v>
-      </c>
-      <c r="I32" t="s">
+      <c r="G34" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H34" t="s">
+        <v>16</v>
+      </c>
+      <c r="I34" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="57.6">
-      <c r="A33" s="10"/>
-      <c r="B33" t="s">
+    <row r="35" spans="1:9" ht="28.8">
+      <c r="A35" s="9"/>
+      <c r="B35" t="s">
+        <v>132</v>
+      </c>
+      <c r="C35" t="s">
         <v>137</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D35" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35" t="s">
         <v>138</v>
       </c>
-      <c r="D33" t="s">
+      <c r="F35" t="s">
+        <v>135</v>
+      </c>
+      <c r="G35" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H35" t="s">
+        <v>16</v>
+      </c>
+      <c r="I35" t="s">
         <v>139</v>
       </c>
-      <c r="E33" t="s">
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="F33" t="s">
+      <c r="B36" t="s">
         <v>141</v>
       </c>
-      <c r="G33" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H33" t="s">
-        <v>16</v>
-      </c>
-      <c r="I33" t="s">
+      <c r="C36" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" ht="28.8">
-      <c r="A34" s="10"/>
-      <c r="B34" t="s">
+      <c r="D36" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" t="s">
         <v>143</v>
       </c>
-      <c r="C34" t="s">
+      <c r="F36" t="s">
         <v>144</v>
       </c>
-      <c r="D34" t="s">
-        <v>13</v>
-      </c>
-      <c r="E34" t="s">
+      <c r="G36" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H36" t="s">
+        <v>16</v>
+      </c>
+      <c r="I36" t="s">
         <v>145</v>
       </c>
-      <c r="F34" t="s">
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="8"/>
+      <c r="B37" t="s">
+        <v>141</v>
+      </c>
+      <c r="C37" t="s">
         <v>146</v>
       </c>
-      <c r="G34" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H34" t="s">
-        <v>16</v>
-      </c>
-      <c r="I34" t="s">
+      <c r="D37" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" ht="28.8">
-      <c r="A35" s="11"/>
-      <c r="B35" t="s">
-        <v>143</v>
-      </c>
-      <c r="C35" t="s">
+      <c r="F37" t="s">
+        <v>144</v>
+      </c>
+      <c r="G37" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H37" t="s">
+        <v>16</v>
+      </c>
+      <c r="I37" t="s">
         <v>148</v>
       </c>
-      <c r="D35" t="s">
-        <v>13</v>
-      </c>
-      <c r="E35" t="s">
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="8"/>
+      <c r="B38" t="s">
+        <v>141</v>
+      </c>
+      <c r="C38" t="s">
         <v>149</v>
       </c>
-      <c r="F35" t="s">
-        <v>146</v>
-      </c>
-      <c r="G35" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H35" t="s">
-        <v>16</v>
-      </c>
-      <c r="I35" t="s">
+      <c r="D38" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="36" spans="1:9">
-      <c r="A36" s="9" t="s">
+      <c r="F38" t="s">
+        <v>144</v>
+      </c>
+      <c r="G38" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I38" t="s">
         <v>151</v>
       </c>
-      <c r="B36" t="s">
+    </row>
+    <row r="39" spans="1:9" ht="43.2">
+      <c r="A39" s="8"/>
+      <c r="B39" t="s">
         <v>152</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C39" t="s">
         <v>153</v>
       </c>
-      <c r="D36" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" t="s">
+      <c r="D39" t="s">
+        <v>13</v>
+      </c>
+      <c r="E39" t="s">
         <v>154</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F39" t="s">
         <v>155</v>
       </c>
-      <c r="G36" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H36" t="s">
-        <v>16</v>
-      </c>
-      <c r="I36" t="s">
+      <c r="G39" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H39" t="s">
+        <v>16</v>
+      </c>
+      <c r="I39" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
-      <c r="A37" s="10"/>
-      <c r="B37" t="s">
+    <row r="40" spans="1:9" ht="28.8">
+      <c r="A40" s="8"/>
+      <c r="B40" t="s">
         <v>152</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C40" t="s">
         <v>157</v>
       </c>
-      <c r="D37" t="s">
-        <v>13</v>
-      </c>
-      <c r="E37" t="s">
+      <c r="D40" t="s">
+        <v>13</v>
+      </c>
+      <c r="E40" t="s">
         <v>158</v>
       </c>
-      <c r="F37" t="s">
-        <v>155</v>
-      </c>
-      <c r="G37" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H37" t="s">
-        <v>16</v>
-      </c>
-      <c r="I37" t="s">
+      <c r="F40" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="38" spans="1:9">
-      <c r="A38" s="10"/>
-      <c r="B38" t="s">
+      <c r="G40" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H40" t="s">
+        <v>16</v>
+      </c>
+      <c r="I40" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="28.8">
+      <c r="A41" s="8"/>
+      <c r="B41" t="s">
         <v>152</v>
       </c>
-      <c r="C38" t="s">
-        <v>160</v>
-      </c>
-      <c r="D38" t="s">
-        <v>13</v>
-      </c>
-      <c r="E38" t="s">
+      <c r="C41" t="s">
         <v>161</v>
       </c>
-      <c r="F38" t="s">
-        <v>155</v>
-      </c>
-      <c r="G38" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H38" t="s">
-        <v>16</v>
-      </c>
-      <c r="I38" t="s">
+      <c r="D41" t="s">
+        <v>13</v>
+      </c>
+      <c r="E41" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" ht="43.2">
-      <c r="A39" s="10"/>
-      <c r="B39" t="s">
+      <c r="F41" t="s">
         <v>163</v>
       </c>
-      <c r="C39" t="s">
+      <c r="G41" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H41" t="s">
+        <v>16</v>
+      </c>
+      <c r="I41" t="s">
         <v>164</v>
       </c>
-      <c r="D39" t="s">
-        <v>13</v>
-      </c>
-      <c r="E39" t="s">
+    </row>
+    <row r="42" spans="1:9" ht="28.8">
+      <c r="A42" s="8"/>
+      <c r="B42" t="s">
         <v>165</v>
       </c>
-      <c r="F39" t="s">
+      <c r="C42" t="s">
         <v>166</v>
       </c>
-      <c r="G39" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H39" t="s">
-        <v>16</v>
-      </c>
-      <c r="I39" t="s">
+      <c r="D42" t="s">
+        <v>13</v>
+      </c>
+      <c r="E42" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" ht="28.8">
-      <c r="A40" s="10"/>
-      <c r="B40" t="s">
-        <v>163</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="F42" t="s">
         <v>168</v>
       </c>
-      <c r="D40" t="s">
-        <v>13</v>
-      </c>
-      <c r="E40" t="s">
+      <c r="G42" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H42" t="s">
+        <v>16</v>
+      </c>
+      <c r="I42" t="s">
         <v>169</v>
       </c>
-      <c r="F40" t="s">
+    </row>
+    <row r="43" spans="1:9" ht="28.8">
+      <c r="A43" s="9"/>
+      <c r="B43" t="s">
         <v>170</v>
       </c>
-      <c r="G40" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H40" t="s">
-        <v>16</v>
-      </c>
-      <c r="I40" t="s">
+      <c r="C43" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" ht="28.8">
-      <c r="A41" s="10"/>
-      <c r="B41" t="s">
-        <v>163</v>
-      </c>
-      <c r="C41" t="s">
+      <c r="D43" t="s">
         <v>172</v>
       </c>
-      <c r="D41" t="s">
-        <v>13</v>
-      </c>
-      <c r="E41" t="s">
+      <c r="E43" t="s">
         <v>173</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F43" t="s">
         <v>174</v>
       </c>
-      <c r="G41" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H41" t="s">
-        <v>16</v>
-      </c>
-      <c r="I41" t="s">
+      <c r="G43" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H43" t="s">
+        <v>16</v>
+      </c>
+      <c r="I43" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="28.8">
-      <c r="A42" s="10"/>
-      <c r="B42" t="s">
+    <row r="44" spans="1:9" ht="43.2">
+      <c r="A44" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="C42" t="s">
+      <c r="B44" t="s">
         <v>177</v>
       </c>
-      <c r="D42" t="s">
-        <v>13</v>
-      </c>
-      <c r="E42" t="s">
+      <c r="C44" t="s">
         <v>178</v>
       </c>
-      <c r="F42" t="s">
+      <c r="D44" t="s">
+        <v>172</v>
+      </c>
+      <c r="E44" t="s">
         <v>179</v>
       </c>
-      <c r="G42" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H42" t="s">
-        <v>16</v>
-      </c>
-      <c r="I42" t="s">
+      <c r="F44" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" ht="28.8">
-      <c r="A43" s="11"/>
-      <c r="B43" t="s">
+      <c r="G44" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H44" t="s">
+        <v>16</v>
+      </c>
+      <c r="I44" t="s">
         <v>181</v>
       </c>
-      <c r="C43" t="s">
+    </row>
+    <row r="45" spans="1:9" ht="28.8">
+      <c r="A45" s="8"/>
+      <c r="B45" t="s">
+        <v>177</v>
+      </c>
+      <c r="C45" t="s">
         <v>182</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D45" t="s">
+        <v>13</v>
+      </c>
+      <c r="E45" t="s">
         <v>183</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F45" t="s">
         <v>184</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G45" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H45" t="s">
+        <v>16</v>
+      </c>
+      <c r="I45" t="s">
         <v>185</v>
       </c>
-      <c r="G43" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H43" t="s">
-        <v>16</v>
-      </c>
-      <c r="I43" t="s">
+    </row>
+    <row r="46" spans="1:9" ht="28.8">
+      <c r="A46" s="8"/>
+      <c r="B46" t="s">
+        <v>177</v>
+      </c>
+      <c r="C46" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" ht="43.2">
-      <c r="A44" s="9" t="s">
+      <c r="D46" t="s">
+        <v>13</v>
+      </c>
+      <c r="E46" t="s">
         <v>187</v>
       </c>
-      <c r="B44" t="s">
+      <c r="F46" t="s">
         <v>188</v>
       </c>
-      <c r="C44" t="s">
+      <c r="G46" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H46" t="s">
+        <v>16</v>
+      </c>
+      <c r="I46" t="s">
         <v>189</v>
       </c>
-      <c r="D44" t="s">
-        <v>183</v>
-      </c>
-      <c r="E44" t="s">
+    </row>
+    <row r="47" spans="1:9" ht="28.8">
+      <c r="A47" s="8"/>
+      <c r="B47" t="s">
+        <v>177</v>
+      </c>
+      <c r="C47" t="s">
         <v>190</v>
       </c>
-      <c r="F44" t="s">
+      <c r="D47" t="s">
+        <v>13</v>
+      </c>
+      <c r="E47" t="s">
         <v>191</v>
       </c>
-      <c r="G44" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H44" t="s">
-        <v>16</v>
-      </c>
-      <c r="I44" t="s">
+      <c r="F47" t="s">
+        <v>184</v>
+      </c>
+      <c r="G47" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H47" t="s">
+        <v>16</v>
+      </c>
+      <c r="I47" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="28.8">
-      <c r="A45" s="10"/>
-      <c r="B45" t="s">
-        <v>188</v>
-      </c>
-      <c r="C45" t="s">
+    <row r="48" spans="1:9" ht="28.8">
+      <c r="A48" s="9"/>
+      <c r="B48" t="s">
         <v>193</v>
       </c>
-      <c r="D45" t="s">
-        <v>13</v>
-      </c>
-      <c r="E45" t="s">
+      <c r="C48" t="s">
         <v>194</v>
       </c>
-      <c r="F45" t="s">
+      <c r="D48" t="s">
         <v>195</v>
       </c>
-      <c r="G45" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H45" t="s">
-        <v>16</v>
-      </c>
-      <c r="I45" t="s">
+      <c r="E48" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" ht="28.8">
-      <c r="A46" s="10"/>
-      <c r="B46" t="s">
-        <v>188</v>
-      </c>
-      <c r="C46" t="s">
+      <c r="F48" t="s">
         <v>197</v>
       </c>
-      <c r="D46" t="s">
-        <v>13</v>
-      </c>
-      <c r="E46" t="s">
+      <c r="G48" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H48" t="s">
+        <v>16</v>
+      </c>
+      <c r="I48" t="s">
         <v>198</v>
       </c>
-      <c r="F46" t="s">
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G46" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H46" t="s">
-        <v>16</v>
-      </c>
-      <c r="I46" t="s">
+      <c r="B49" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" ht="28.8">
-      <c r="A47" s="10"/>
-      <c r="B47" t="s">
-        <v>188</v>
-      </c>
-      <c r="C47" t="s">
+      <c r="C49" t="s">
         <v>201</v>
       </c>
-      <c r="D47" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" t="s">
+      <c r="D49" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" t="s">
         <v>202</v>
       </c>
-      <c r="F47" t="s">
-        <v>195</v>
-      </c>
-      <c r="G47" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H47" t="s">
-        <v>16</v>
-      </c>
-      <c r="I47" t="s">
+      <c r="F49" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" ht="28.8">
-      <c r="A48" s="11"/>
-      <c r="B48" t="s">
+      <c r="G49" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H49" t="s">
+        <v>16</v>
+      </c>
+      <c r="I49" t="s">
         <v>204</v>
       </c>
-      <c r="C48" t="s">
+    </row>
+    <row r="50" spans="1:9" ht="28.8">
+      <c r="A50" s="8"/>
+      <c r="B50" t="s">
+        <v>200</v>
+      </c>
+      <c r="C50" t="s">
         <v>205</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" t="s">
         <v>206</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F50" t="s">
         <v>207</v>
       </c>
-      <c r="F48" t="s">
+      <c r="G50" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H50" t="s">
+        <v>16</v>
+      </c>
+      <c r="I50" t="s">
         <v>208</v>
       </c>
-      <c r="G48" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H48" t="s">
-        <v>16</v>
-      </c>
-      <c r="I48" t="s">
+    </row>
+    <row r="51" spans="1:9" ht="28.8">
+      <c r="A51" s="8"/>
+      <c r="B51" t="s">
+        <v>200</v>
+      </c>
+      <c r="C51" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="49" spans="1:9">
-      <c r="A49" s="9" t="s">
+      <c r="D51" t="s">
+        <v>13</v>
+      </c>
+      <c r="E51" t="s">
         <v>210</v>
       </c>
-      <c r="B49" t="s">
+      <c r="F51" t="s">
+        <v>207</v>
+      </c>
+      <c r="G51" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H51" t="s">
+        <v>16</v>
+      </c>
+      <c r="I51" t="s">
         <v>211</v>
       </c>
-      <c r="C49" t="s">
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="8"/>
+      <c r="B52" t="s">
         <v>212</v>
       </c>
-      <c r="D49" t="s">
-        <v>13</v>
-      </c>
-      <c r="E49" t="s">
+      <c r="C52" t="s">
         <v>213</v>
       </c>
-      <c r="F49" t="s">
+      <c r="D52" t="s">
+        <v>13</v>
+      </c>
+      <c r="E52" t="s">
         <v>214</v>
       </c>
-      <c r="G49" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H49" t="s">
-        <v>16</v>
-      </c>
-      <c r="I49" t="s">
+      <c r="F52" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" ht="28.8">
-      <c r="A50" s="10"/>
-      <c r="B50" t="s">
-        <v>211</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="G52" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H52" t="s">
+        <v>16</v>
+      </c>
+      <c r="I52" t="s">
         <v>216</v>
       </c>
-      <c r="D50" t="s">
-        <v>13</v>
-      </c>
-      <c r="E50" t="s">
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="8"/>
+      <c r="B53" t="s">
         <v>217</v>
       </c>
-      <c r="F50" t="s">
+      <c r="C53" t="s">
         <v>218</v>
       </c>
-      <c r="G50" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H50" t="s">
-        <v>16</v>
-      </c>
-      <c r="I50" t="s">
+      <c r="D53" t="s">
+        <v>13</v>
+      </c>
+      <c r="E53" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" ht="28.8">
-      <c r="A51" s="10"/>
-      <c r="B51" t="s">
-        <v>211</v>
-      </c>
-      <c r="C51" t="s">
+      <c r="F53" t="s">
         <v>220</v>
       </c>
-      <c r="D51" t="s">
-        <v>13</v>
-      </c>
-      <c r="E51" t="s">
+      <c r="G53" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H53" t="s">
+        <v>16</v>
+      </c>
+      <c r="I53" t="s">
         <v>221</v>
       </c>
-      <c r="F51" t="s">
-        <v>218</v>
-      </c>
-      <c r="G51" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H51" t="s">
-        <v>16</v>
-      </c>
-      <c r="I51" t="s">
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="9"/>
+      <c r="B54" t="s">
+        <v>217</v>
+      </c>
+      <c r="C54" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="52" spans="1:9">
-      <c r="A52" s="10"/>
-      <c r="B52" t="s">
+      <c r="D54" t="s">
+        <v>13</v>
+      </c>
+      <c r="E54" t="s">
         <v>223</v>
       </c>
-      <c r="C52" t="s">
+      <c r="F54" t="s">
+        <v>220</v>
+      </c>
+      <c r="G54" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H54" t="s">
+        <v>16</v>
+      </c>
+      <c r="I54" t="s">
         <v>224</v>
       </c>
-      <c r="D52" t="s">
-        <v>13</v>
-      </c>
-      <c r="E52" t="s">
+    </row>
+    <row r="55" spans="1:9" ht="28.8">
+      <c r="A55" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="F52" t="s">
+      <c r="B55" t="s">
         <v>226</v>
       </c>
-      <c r="G52" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H52" t="s">
-        <v>16</v>
-      </c>
-      <c r="I52" t="s">
+      <c r="C55" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="53" spans="1:9">
-      <c r="A53" s="10"/>
-      <c r="B53" t="s">
+      <c r="D55" t="s">
+        <v>13</v>
+      </c>
+      <c r="E55" t="s">
         <v>228</v>
       </c>
-      <c r="C53" t="s">
+      <c r="F55" t="s">
+        <v>30</v>
+      </c>
+      <c r="G55" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H55" t="s">
+        <v>16</v>
+      </c>
+      <c r="I55" t="s">
         <v>229</v>
       </c>
-      <c r="D53" t="s">
-        <v>13</v>
-      </c>
-      <c r="E53" t="s">
+    </row>
+    <row r="56" spans="1:9" ht="28.8">
+      <c r="A56" s="8"/>
+      <c r="B56" t="s">
+        <v>226</v>
+      </c>
+      <c r="C56" t="s">
         <v>230</v>
       </c>
-      <c r="F53" t="s">
+      <c r="D56" t="s">
+        <v>13</v>
+      </c>
+      <c r="E56" t="s">
         <v>231</v>
       </c>
-      <c r="G53" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H53" t="s">
-        <v>16</v>
-      </c>
-      <c r="I53" t="s">
+      <c r="F56" t="s">
+        <v>46</v>
+      </c>
+      <c r="G56" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H56" t="s">
+        <v>16</v>
+      </c>
+      <c r="I56" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="54" spans="1:9">
-      <c r="A54" s="11"/>
-      <c r="B54" t="s">
-        <v>228</v>
-      </c>
-      <c r="C54" t="s">
+    <row r="57" spans="1:9">
+      <c r="A57" s="8"/>
+      <c r="B57" t="s">
+        <v>226</v>
+      </c>
+      <c r="C57" t="s">
         <v>233</v>
       </c>
-      <c r="D54" t="s">
-        <v>13</v>
-      </c>
-      <c r="E54" t="s">
+      <c r="D57" t="s">
+        <v>13</v>
+      </c>
+      <c r="E57" t="s">
         <v>234</v>
       </c>
-      <c r="F54" t="s">
-        <v>231</v>
-      </c>
-      <c r="G54" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H54" t="s">
-        <v>16</v>
-      </c>
-      <c r="I54" t="s">
+      <c r="F57" t="s">
+        <v>35</v>
+      </c>
+      <c r="G57" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H57" t="s">
+        <v>16</v>
+      </c>
+      <c r="I57" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="28.8">
-      <c r="A55" s="9" t="s">
+    <row r="58" spans="1:9">
+      <c r="A58" s="8"/>
+      <c r="B58" t="s">
         <v>236</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C58" t="s">
         <v>237</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D58" t="s">
+        <v>13</v>
+      </c>
+      <c r="E58" t="s">
         <v>238</v>
       </c>
-      <c r="D55" t="s">
-        <v>13</v>
-      </c>
-      <c r="E55" t="s">
+      <c r="F58" t="s">
+        <v>59</v>
+      </c>
+      <c r="G58" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H58" t="s">
+        <v>16</v>
+      </c>
+      <c r="I58" t="s">
         <v>239</v>
       </c>
-      <c r="F55" t="s">
-        <v>32</v>
-      </c>
-      <c r="G55" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H55" t="s">
-        <v>16</v>
-      </c>
-      <c r="I55" t="s">
+    </row>
+    <row r="59" spans="1:9" ht="28.8">
+      <c r="A59" s="8"/>
+      <c r="B59" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" ht="28.8">
-      <c r="A56" s="10"/>
-      <c r="B56" t="s">
-        <v>237</v>
-      </c>
-      <c r="C56" t="s">
+      <c r="C59" t="s">
         <v>241</v>
       </c>
-      <c r="D56" t="s">
-        <v>13</v>
-      </c>
-      <c r="E56" t="s">
+      <c r="D59" t="s">
+        <v>13</v>
+      </c>
+      <c r="E59" t="s">
         <v>242</v>
       </c>
-      <c r="F56" t="s">
-        <v>49</v>
-      </c>
-      <c r="G56" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H56" t="s">
-        <v>16</v>
-      </c>
-      <c r="I56" t="s">
+      <c r="F59" t="s">
+        <v>87</v>
+      </c>
+      <c r="G59" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H59" t="s">
+        <v>16</v>
+      </c>
+      <c r="I59" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="57" spans="1:9">
-      <c r="A57" s="10"/>
-      <c r="B57" t="s">
-        <v>237</v>
-      </c>
-      <c r="C57" t="s">
+    <row r="60" spans="1:9" ht="28.8">
+      <c r="A60" s="9"/>
+      <c r="B60" t="s">
         <v>244</v>
       </c>
-      <c r="D57" t="s">
-        <v>13</v>
-      </c>
-      <c r="E57" t="s">
+      <c r="C60" t="s">
         <v>245</v>
       </c>
-      <c r="F57" t="s">
-        <v>37</v>
-      </c>
-      <c r="G57" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H57" t="s">
-        <v>16</v>
-      </c>
-      <c r="I57" t="s">
+      <c r="D60" t="s">
+        <v>13</v>
+      </c>
+      <c r="E60" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="58" spans="1:9">
-      <c r="A58" s="10"/>
-      <c r="B58" t="s">
+      <c r="F60" t="s">
+        <v>207</v>
+      </c>
+      <c r="G60" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H60" t="s">
+        <v>16</v>
+      </c>
+      <c r="I60" t="s">
         <v>247</v>
-      </c>
-      <c r="C58" t="s">
-        <v>248</v>
-      </c>
-      <c r="D58" t="s">
-        <v>13</v>
-      </c>
-      <c r="E58" t="s">
-        <v>249</v>
-      </c>
-      <c r="F58" t="s">
-        <v>64</v>
-      </c>
-      <c r="G58" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H58" t="s">
-        <v>16</v>
-      </c>
-      <c r="I58" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="28.8">
-      <c r="A59" s="10"/>
-      <c r="B59" t="s">
-        <v>251</v>
-      </c>
-      <c r="C59" t="s">
-        <v>252</v>
-      </c>
-      <c r="D59" t="s">
-        <v>13</v>
-      </c>
-      <c r="E59" t="s">
-        <v>253</v>
-      </c>
-      <c r="F59" t="s">
-        <v>97</v>
-      </c>
-      <c r="G59" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H59" t="s">
-        <v>16</v>
-      </c>
-      <c r="I59" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="28.8">
-      <c r="A60" s="11"/>
-      <c r="B60" t="s">
-        <v>255</v>
-      </c>
-      <c r="C60" t="s">
-        <v>256</v>
-      </c>
-      <c r="D60" t="s">
-        <v>13</v>
-      </c>
-      <c r="E60" t="s">
-        <v>257</v>
-      </c>
-      <c r="F60" t="s">
-        <v>218</v>
-      </c>
-      <c r="G60" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="H60" t="s">
-        <v>16</v>
-      </c>
-      <c r="I60" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="28.8">
       <c r="A61" s="3" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>1</v>
@@ -3073,27 +3170,27 @@
         <v>1</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
     </row>
     <row r="117" spans="1:9">
-      <c r="A117" s="12" t="s">
-        <v>259</v>
+      <c r="A117" s="10" t="s">
+        <v>248</v>
       </c>
       <c r="B117" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="C117" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="D117" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="E117" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="F117" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="G117" s="2">
         <v>4</v>
@@ -3102,25 +3199,25 @@
         <v>16</v>
       </c>
       <c r="I117" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
     </row>
     <row r="118" spans="1:9">
-      <c r="A118" s="13"/>
+      <c r="A118" s="11"/>
       <c r="B118" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="C118" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="D118" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="E118" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="F118" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="G118" s="2">
         <v>4</v>
@@ -3129,25 +3226,25 @@
         <v>16</v>
       </c>
       <c r="I118" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
     </row>
     <row r="119" spans="1:9">
-      <c r="A119" s="13"/>
+      <c r="A119" s="11"/>
       <c r="B119" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="C119" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="D119" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="E119" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="F119" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="G119" s="2">
         <v>2</v>
@@ -3156,25 +3253,25 @@
         <v>16</v>
       </c>
       <c r="I119" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
     </row>
     <row r="120" spans="1:9">
-      <c r="A120" s="13"/>
+      <c r="A120" s="11"/>
       <c r="B120" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="C120" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="D120" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="E120" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="F120" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="G120" s="2">
         <v>2</v>
@@ -3183,25 +3280,25 @@
         <v>16</v>
       </c>
       <c r="I120" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
     </row>
     <row r="121" spans="1:9">
-      <c r="A121" s="14"/>
+      <c r="A121" s="12"/>
       <c r="B121" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="C121" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="D121" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="E121" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="F121" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="G121" s="2">
         <v>12</v>
@@ -3210,21 +3307,21 @@
         <v>16</v>
       </c>
       <c r="I121" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:A9"/>
+    <mergeCell ref="A10:A19"/>
+    <mergeCell ref="A21:A27"/>
+    <mergeCell ref="A28:A35"/>
     <mergeCell ref="A44:A48"/>
     <mergeCell ref="A49:A54"/>
     <mergeCell ref="A55:A60"/>
     <mergeCell ref="A117:A121"/>
     <mergeCell ref="A36:A43"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:A9"/>
-    <mergeCell ref="A10:A19"/>
-    <mergeCell ref="A21:A27"/>
-    <mergeCell ref="A28:A35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>